<commit_message>
mis a jour btn de tableau
</commit_message>
<xml_diff>
--- a/assets/TABLEAU_DE_SYNTHESE_BTS_SIO_2026.xlsx
+++ b/assets/TABLEAU_DE_SYNTHESE_BTS_SIO_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WEB DEVELOPEMENT\sigma course\Protfilo_updated_site\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{309C182A-6B20-468F-9240-AE9BC97BDB3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0DABFCA-9E4F-44CE-88BA-3DF1C3A9E1BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -191,7 +191,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -253,6 +253,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -665,7 +671,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -760,9 +766,48 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -787,44 +832,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1238,56 +1247,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="32"/>
+      <c r="H1" s="34"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="32" t="s">
+      <c r="A2" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="39" t="s">
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="34"/>
-      <c r="H3" s="40"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="53"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="49" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="38"/>
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="51"/>
       <c r="F4" s="16" t="s">
         <v>8</v>
       </c>
@@ -1299,22 +1308,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="52"/>
-      <c r="H5" s="53"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="45"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="49" t="s">
+      <c r="B6" s="41" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1337,8 +1346,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="42"/>
-      <c r="B7" s="50"/>
+      <c r="A7" s="33"/>
+      <c r="B7" s="42"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1394,16 +1403,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="44"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="45"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="37"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1500,7 +1509,7 @@
       <c r="D10" s="18"/>
       <c r="E10" s="18"/>
       <c r="F10" s="18"/>
-      <c r="G10" s="27"/>
+      <c r="G10" s="29"/>
       <c r="H10" s="28"/>
       <c r="I10"/>
       <c r="J10"/>
@@ -1550,7 +1559,7 @@
       <c r="E11" s="18"/>
       <c r="F11" s="27"/>
       <c r="G11" s="27"/>
-      <c r="H11" s="19"/>
+      <c r="H11" s="28"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1648,7 +1657,7 @@
       <c r="E13" s="27"/>
       <c r="F13" s="27"/>
       <c r="G13" s="27"/>
-      <c r="H13" s="19"/>
+      <c r="H13" s="28"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1697,7 +1706,7 @@
       <c r="E14" s="18"/>
       <c r="F14" s="27"/>
       <c r="G14" s="27"/>
-      <c r="H14" s="19"/>
+      <c r="H14" s="54"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1915,16 +1924,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="46" t="s">
+      <c r="A19" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="47"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="47"/>
-      <c r="E19" s="47"/>
-      <c r="F19" s="47"/>
-      <c r="G19" s="47"/>
-      <c r="H19" s="48"/>
+      <c r="B19" s="39"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="40"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -2277,16 +2286,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="46" t="s">
+      <c r="A27" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="47"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="48"/>
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="40"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2743,6 +2752,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2750,11 +2764,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>